<commit_message>
Add apps: WJacobsonGalan EGriffith
</commit_message>
<xml_diff>
--- a/nhfp-apps/nhfp-apps.xlsx
+++ b/nhfp-apps/nhfp-apps.xlsx
@@ -69,12 +69,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDEDF2"/>
+        <fgColor rgb="00EFF9FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EFF9FB"/>
+        <fgColor rgb="00FDEDF2"/>
       </patternFill>
     </fill>
     <fill>
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -777,19 +777,19 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Jaren Ashcraft</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
+            <t>Emily Griffith</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
           </r>
           <r>
             <rPr>
@@ -801,62 +801,62 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>The Milky Way and Resolved Stellar Populations</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Beyond Mg and Fe: Exploring Detailed Nucleosynthetic Patterns</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Wynn Jacobson-Galan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Optimizing The Vector Field For Next-Generation Astrophysics</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Andrew Saydjari</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>The Milky Way and Resolved Stellar Populations</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Inferring Kinematic and Chemical Maps of Galactic Dust</t>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Stellar Physics</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Final Moments: Uncovering the Rate of Enhanced Red Supergiant Mass-loss in the Local Volume</t>
         </is>
       </c>
     </row>
@@ -867,19 +867,19 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Adam Smercina</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
+            <t>Jaren Ashcraft</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
           </r>
           <r>
             <rPr>
@@ -896,57 +896,57 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Optimizing The Vector Field For Next-Generation Astrophysics</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Andrew Saydjari</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
           <t>The Milky Way and Resolved Stellar Populations</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>A Portrait of the Triangulum: Advancing a New Frontier of Galaxy Evolution with Resolved Stars</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Sylvia Biscoveanu</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Gravitational Wave Astrophysics</t>
-        </is>
-      </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>From black holes to the Big Bang: astrophysics and cosmology with gravitational waves and their electromagnetic counterparts</t>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Inferring Kinematic and Chemical Maps of Galactic Dust</t>
         </is>
       </c>
     </row>
@@ -957,6 +957,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Adam Smercina</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>The Milky Way and Resolved Stellar Populations</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>A Portrait of the Triangulum: Advancing a New Frontier of Galaxy Evolution with Resolved Stars</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Sylvia Biscoveanu</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Gravitational Wave Astrophysics</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>From black holes to the Big Bang: astrophysics and cosmology with gravitational waves and their electromagnetic counterparts</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Maggie Thompson</t>
           </r>
           <r>
@@ -979,24 +1069,24 @@
           </r>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>To Explore Strange New Worlds: Connecting the Interiors and Atmospheres of Rocky Exoplanets</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1024,24 +1114,24 @@
           </r>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>Leveraging HST for a New Era of Precision NIR SN Ia Cosmology</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1069,24 +1159,24 @@
           </r>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>The Evolution of Young Exoplanet Atmospheres in the Presence of Extreme Stellar Activity</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1114,24 +1204,24 @@
           </r>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>Illuminating the Primeval Universe with Lyman$\alpha$</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1159,109 +1249,19 @@
           </r>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Constraining Post-main-sequence Angular Momentum Evolution with Mixed-mode Asteroseismology</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Dávid Guszejnov</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Stellar Physics</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>The Role of Physical Processes and the Environment in Star Formation</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Pradip Gatkine</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D17" s="15" t="inlineStr">
-        <is>
-          <t>Probing the CGM-galaxy connection using Multi-object Spectroscopy and Astrophotonics</t>
         </is>
       </c>
     </row>
@@ -1272,6 +1272,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Dávid Guszejnov</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Stellar Physics</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>The Role of Physical Processes and the Environment in Star Formation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Pradip Gatkine</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Probing the CGM-galaxy connection using Multi-object Spectroscopy and Astrophotonics</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Michael Grudić</t>
           </r>
           <r>
@@ -1294,24 +1384,24 @@
           </r>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>Star-Formation Physics from Cosmos to Cores</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1339,24 +1429,24 @@
           </r>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Atmospheres as Windows to the Diversity of Extrasolar Planets</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1384,24 +1474,24 @@
           </r>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>Internal Structure of Massive Elliptical Galaxies: The Missing Piece at the Intersection of Astrophysics and Cosmology</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1429,24 +1519,24 @@
           </r>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Cosmic Ray Diffusion in the Multi-phase Interstellar Medium</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1474,24 +1564,24 @@
           </r>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>Exoplanet Formation and Protoplanetary Disks</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>Formation and Dynamics of Short-Period Exoplanetary Systems</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1519,24 +1609,24 @@
           </r>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>The Role of Aerosols in the Formation and Early Evolution of Giant Planets</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1564,24 +1654,24 @@
           </r>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>Gravitational Wave Astrophysics</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Deciphering the Biography of Massive Stars: Compact Object Mergers as a Rosetta Stone</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1609,24 +1699,24 @@
           </r>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>A New Era of Exoplanet Imaging Mid-Infrared Exploration of the Habitable Zones of Nearby Stars</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1654,109 +1744,19 @@
           </r>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Two Projects with Circumbinary Planets—Using the Planets to Solve Super-Earth Formation, and the Binaries to Empirically Constrain M-dwarfs</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>David Jones</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>Physics and Cosmology</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>Supernova Cosmology in the Era of Cosmological Tensions</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Arpita Roy</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>Of Worlds to Come: Delivering On the Promise of Extreme Precision Spectroscopy for Exoplanets</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Yao-Yuan Mao</t>
+            <t>David Jones</t>
           </r>
           <r>
             <rPr>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>The Galaxy–Halo Connection: Probing the Dark Universe with Galaxies</t>
+          <t>Supernova Cosmology in the Era of Cosmological Tensions</t>
         </is>
       </c>
     </row>
@@ -1812,19 +1812,19 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Georgia Panopoulou</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
+            <t>Arpita Roy</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
           </r>
           <r>
             <rPr>
@@ -1836,17 +1836,17 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>The Milky Way and Resolved Stellar Populations</t>
+          <t>Exoplanets and Habitability</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>A unique approach to the determination of the Galactic magnetic field using starlight and synchrotron polarization observations</t>
+          <t>Of Worlds to Come: Delivering On the Promise of Extreme Precision Spectroscopy for Exoplanets</t>
         </is>
       </c>
     </row>
@@ -1857,6 +1857,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Yao-Yuan Mao</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Physics and Cosmology</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>The Galaxy–Halo Connection: Probing the Dark Universe with Galaxies</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Georgia Panopoulou</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>The Milky Way and Resolved Stellar Populations</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>A unique approach to the determination of the Galactic magnetic field using starlight and synchrotron polarization observations</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Dillon Brout</t>
           </r>
           <r>
@@ -1879,24 +1969,24 @@
           </r>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Improving Cosmological Constraints with the Dark Energy Survey Supernova Program and a Decade of Type Ia Supernovae</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1924,24 +2014,24 @@
           </r>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>The Milky Way and Resolved Stellar Populations</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>Ultra-High Resolution Simulations of the Milky Way and its Satellites</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1969,24 +2059,24 @@
           </r>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Planetary Collisions around Low-Mass Stars: Constraining the Timescale for Collisions and Testing the Origin of the Kepler Dichotomy</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2014,24 +2104,24 @@
           </r>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Subgiants: Models, Rotation, Convection, and Planets</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2059,24 +2149,24 @@
           </r>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr">
+      <c r="C37" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>Revolutionizing Reionization with JWST</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2104,24 +2194,24 @@
           </r>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>Mapping the true boundary of dark matter halos with the splashback radius</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2149,109 +2239,19 @@
           </r>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="C37" s="12" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D37" s="13" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>The Role of Neutral‐ion Coupling in Star Formation</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Raphaelle Haywood</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>Breaking the Ultimate Barrier to Characterizing Other Earths</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Johanna Teske</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>Characterizing the Diversity of Small Planet Compositions via Planet Densities and Host Star Abundances</t>
         </is>
       </c>
     </row>
@@ -2262,6 +2262,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Raphaelle Haywood</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Breaking the Ultimate Barrier to Characterizing Other Earths</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Johanna Teske</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Characterizing the Diversity of Small Planet Compositions via Planet Densities and Host Star Abundances</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Brett McGuire</t>
           </r>
           <r>
@@ -2284,109 +2374,19 @@
           </r>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>The Milky Way and Resolved Stellar Populations</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="D42" s="7" t="inlineStr">
         <is>
           <t>Getting Away from One-Pot Syntheses: Heterogeneity in Molecular Evolution Revealed with ALMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Andrew Vanderburg</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>The Galactic Distribution of Exoplanets</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Sean Johnson</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
-      </c>
-      <c r="C42" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>Unveiling the relationship between AGN and the CGM: feeding and feedback</t>
         </is>
       </c>
     </row>
@@ -2397,6 +2397,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Andrew Vanderburg</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>The Galactic Distribution of Exoplanets</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Sean Johnson</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>Unveiling the relationship between AGN and the CGM: feeding and feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Lia Corrales</t>
           </r>
           <r>
@@ -2419,24 +2509,24 @@
           </r>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>The Milky Way and Resolved Stellar Populations</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D45" s="7" t="inlineStr">
         <is>
           <t>Bringing the Galactic Center into focus with dust scattering</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2464,24 +2554,24 @@
           </r>
         </is>
       </c>
-      <c r="B44" s="16" t="inlineStr">
+      <c r="B46" s="16" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="C44" s="16" t="inlineStr">
+      <c r="C46" s="16" t="inlineStr">
         <is>
           <t>Exoplanet Formation and Protoplanetary Disks</t>
         </is>
       </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="D46" s="17" t="inlineStr">
         <is>
           <t>Finding and Characterizing Forming Protoplanets with Next Generation Adaptive Optics Systems</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2509,24 +2599,24 @@
           </r>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>The Stellar Remnants of Double White Dwarf Mergers</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2554,24 +2644,24 @@
           </r>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C48" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D48" s="9" t="inlineStr">
         <is>
           <t>Characterizing Small Planets Around Bright Stars</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2599,109 +2689,19 @@
           </r>
         </is>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B49" s="8" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D49" s="9" t="inlineStr">
         <is>
           <t>Bridging the Theory Gap: Developing a Novel Cloud Model for Exoplanets</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Peter Behroozi</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B48" s="14" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
-      <c r="C48" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>Uncovering Connections between Galaxy and Dark Matter Halo Assembly Histories</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Daniel Foreman-Mackey</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>(unspecified title)</t>
         </is>
       </c>
     </row>
@@ -2712,6 +2712,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Peter Behroozi</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>Uncovering Connections between Galaxy and Dark Matter Halo Assembly Histories</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Daniel Foreman-Mackey</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>(unspecified title)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Brooke Simmons</t>
           </r>
           <r>
@@ -2734,24 +2824,24 @@
           </r>
         </is>
       </c>
-      <c r="B50" s="14" t="inlineStr">
+      <c r="B52" s="14" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="C50" s="14" t="inlineStr">
+      <c r="C52" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="D52" s="15" t="inlineStr">
         <is>
           <t>Illuminating the Black Hole-Galaxy Connection</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2779,24 +2869,24 @@
           </r>
         </is>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="C51" s="12" t="inlineStr">
+      <c r="C53" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D51" s="13" t="inlineStr">
+      <c r="D53" s="13" t="inlineStr">
         <is>
           <t>From a Detection to Astrophysics in 21 cm Cosmology</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2824,24 +2914,24 @@
           </r>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C54" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D54" s="9" t="inlineStr">
         <is>
           <t>Pushing forward the frontiers of exoplanet characterization</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="16" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2869,24 +2959,24 @@
           </r>
         </is>
       </c>
-      <c r="B53" s="16" t="inlineStr">
+      <c r="B55" s="16" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="C53" s="16" t="inlineStr">
+      <c r="C55" s="16" t="inlineStr">
         <is>
           <t>Exoplanet Formation and Protoplanetary Disks</t>
         </is>
       </c>
-      <c r="D53" s="17" t="inlineStr">
+      <c r="D55" s="17" t="inlineStr">
         <is>
           <t>Formation and evolution of exoplanets</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2914,109 +3004,19 @@
           </r>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C56" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D54" s="7" t="inlineStr">
+      <c r="D56" s="9" t="inlineStr">
         <is>
           <t>Spectroscopy and Cartography of Cool Extrasolar Atmospheres</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Grant Tremblay</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Compact Objects and Accretion</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>Unifying Chandra with ALMA: Star Formation amid Kinematic Black Hole Feedback</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="10" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Francois Foucart</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="C56" s="10" t="inlineStr">
-        <is>
-          <t>Gravitational Wave Astrophysics</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="inlineStr">
-        <is>
-          <t>Simulating compact binary mergers for multi-messenger astronomy</t>
         </is>
       </c>
     </row>
@@ -3027,6 +3027,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Grant Tremblay</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Compact Objects and Accretion</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Unifying Chandra with ALMA: Star Formation amid Kinematic Black Hole Feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Francois Foucart</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>Gravitational Wave Astrophysics</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Simulating compact binary mergers for multi-messenger astronomy</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Krzysztof Nalewajko</t>
           </r>
           <r>
@@ -3049,109 +3139,19 @@
           </r>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Compact Objects and Accretion</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>Understanding Gamma-Ray Flares of Blazars</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Jonathan Trump</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B58" s="14" t="inlineStr">
-        <is>
-          <t>2013</t>
-        </is>
-      </c>
-      <c r="C58" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D58" s="15" t="inlineStr">
-        <is>
-          <t>The Physics Behind Galaxy / Black Hole Coevolution</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Laura Blecha</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B59" s="14" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="C59" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D59" s="15" t="inlineStr">
-        <is>
-          <t>Seeking the Origins of Single and Double Active Black Holes</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,52 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Julie Hlavacek-Larrondo</t>
+            <t>Jonathan Trump</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>The Physics Behind Galaxy / Black Hole Coevolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Laura Blecha</t>
           </r>
           <r>
             <rPr>
@@ -3184,64 +3229,19 @@
           </r>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>2012</t>
         </is>
       </c>
-      <c r="C60" s="14" t="inlineStr">
+      <c r="C61" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D60" s="15" t="inlineStr">
-        <is>
-          <t>Unravelling AGN feedback: from isolated elliptical galaxies to massive clusters of galaxies</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Ann-Marie Madigan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>Stellar Physics</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>The dynamics of stars in disks around massive black holes</t>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>Seeking the Origins of Single and Double Active Black Holes</t>
         </is>
       </c>
     </row>
@@ -3252,6 +3252,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Julie Hlavacek-Larrondo</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>Unravelling AGN feedback: from isolated elliptical galaxies to massive clusters of galaxies</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Ann-Marie Madigan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Stellar Physics</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>The dynamics of stars in disks around massive black holes</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Steven Finkelstein</t>
           </r>
           <r>
@@ -3274,24 +3364,24 @@
           </r>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B64" s="14" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C62" s="14" t="inlineStr">
+      <c r="C64" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D62" s="15" t="inlineStr">
+      <c r="D64" s="15" t="inlineStr">
         <is>
           <t>Measuring the Evolution of Galaxy Physical Properties from z = 2 – 8</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3319,24 +3409,24 @@
           </r>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Compact Objects and Accretion</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>Probing extremes of binary evolution using subluminous X-ray binaries</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3364,24 +3454,24 @@
           </r>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Compact Objects and Accretion</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Theoretical Investigations of Type Ia Supernova Progenitors</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="16" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3409,24 +3499,24 @@
           </r>
         </is>
       </c>
-      <c r="B65" s="16" t="inlineStr">
+      <c r="B67" s="16" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C65" s="16" t="inlineStr">
+      <c r="C67" s="16" t="inlineStr">
         <is>
           <t>Exoplanet Formation and Protoplanetary Disks</t>
         </is>
       </c>
-      <c r="D65" s="17" t="inlineStr">
+      <c r="D67" s="17" t="inlineStr">
         <is>
           <t>The Formation and Structure of Proto-Planetary Disks Around the Youngest Protostars</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3454,24 +3544,24 @@
           </r>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C68" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D66" s="7" t="inlineStr">
+      <c r="D68" s="9" t="inlineStr">
         <is>
           <t>A Search for Exomoons</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="14" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3499,24 +3589,24 @@
           </r>
         </is>
       </c>
-      <c r="B67" s="14" t="inlineStr">
+      <c r="B69" s="14" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="C67" s="14" t="inlineStr">
+      <c r="C69" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D67" s="15" t="inlineStr">
+      <c r="D69" s="15" t="inlineStr">
         <is>
           <t>Revealing Cluster Astrophysics and Evolution with MUSTANG</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="12" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3544,24 +3634,24 @@
           </r>
         </is>
       </c>
-      <c r="B68" s="12" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="C68" s="12" t="inlineStr">
+      <c r="C70" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D68" s="13" t="inlineStr">
+      <c r="D70" s="13" t="inlineStr">
         <is>
           <t>Exploiting Gravitational Wave Observations: Modeling of Extreme-Mass Ratio Inspirals and Tests of Fundamental Physics</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3589,24 +3679,24 @@
           </r>
         </is>
       </c>
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B71" s="8" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C71" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D69" s="7" t="inlineStr">
+      <c r="D71" s="9" t="inlineStr">
         <is>
           <t>(unspecified title)</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="6" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3634,24 +3724,24 @@
           </r>
         </is>
       </c>
-      <c r="B70" s="6" t="inlineStr">
+      <c r="B72" s="8" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="C70" s="6" t="inlineStr">
+      <c r="C72" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D70" s="7" t="inlineStr">
+      <c r="D72" s="9" t="inlineStr">
         <is>
           <t>Dynamical Architecture of Planetary Systems</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3679,109 +3769,19 @@
           </r>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>2009</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>The Angular Diameters and Physical Properties of Low-Mass Stars</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Shelley Wright</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B72" s="14" t="inlineStr">
-        <is>
-          <t>2009</t>
-        </is>
-      </c>
-      <c r="C72" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D72" s="15" t="inlineStr">
-        <is>
-          <t>Galactic Disk Formation, AGN, and Metallicity in the Early Universe: Spatially Resolved Spectroscopy of High-Redshift Galaxies</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Kristian Finlator</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B73" s="14" t="inlineStr">
-        <is>
-          <t>2009</t>
-        </is>
-      </c>
-      <c r="C73" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D73" s="15" t="inlineStr">
-        <is>
-          <t>Radiative Hydrodynamic Simulations of Galaxies in the Reionization Epoch</t>
         </is>
       </c>
     </row>
@@ -3792,6 +3792,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Shelley Wright</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>Galactic Disk Formation, AGN, and Metallicity in the Early Universe: Spatially Resolved Spectroscopy of High-Redshift Galaxies</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Kristian Finlator</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>Radiative Hydrodynamic Simulations of Galaxies in the Reionization Epoch</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>John Wise</t>
           </r>
           <r>
@@ -3814,24 +3904,24 @@
           </r>
         </is>
       </c>
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B76" s="14" t="inlineStr">
         <is>
           <t>2009</t>
         </is>
       </c>
-      <c r="C74" s="14" t="inlineStr">
+      <c r="C76" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D74" s="15" t="inlineStr">
+      <c r="D76" s="15" t="inlineStr">
         <is>
           <t>Ab Initio Dwarf Galaxy Formation – Predictions for JWST and ALMA</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="6" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3859,24 +3949,24 @@
           </r>
         </is>
       </c>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="B77" s="8" t="inlineStr">
         <is>
           <t>2009</t>
         </is>
       </c>
-      <c r="C75" s="6" t="inlineStr">
+      <c r="C77" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D75" s="7" t="inlineStr">
+      <c r="D77" s="9" t="inlineStr">
         <is>
           <t>(unspecified title)</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="4" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3904,24 +3994,24 @@
           </r>
         </is>
       </c>
-      <c r="B76" s="4" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>2007</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D76" s="5" t="inlineStr">
+      <c r="D78" s="5" t="inlineStr">
         <is>
           <t>Nearby, Young Brown Dwarfs: A Comprehensive Study</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="6" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3949,24 +4039,24 @@
           </r>
         </is>
       </c>
-      <c r="B77" s="6" t="inlineStr">
+      <c r="B79" s="8" t="inlineStr">
         <is>
           <t>2007</t>
         </is>
       </c>
-      <c r="C77" s="6" t="inlineStr">
+      <c r="C79" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D77" s="7" t="inlineStr">
+      <c r="D79" s="9" t="inlineStr">
         <is>
           <t>Dynamical detection and migration of multiple-body planetary systems</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="12" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3994,24 +4084,24 @@
           </r>
         </is>
       </c>
-      <c r="B78" s="12" t="inlineStr">
+      <c r="B80" s="12" t="inlineStr">
         <is>
           <t>2006</t>
         </is>
       </c>
-      <c r="C78" s="12" t="inlineStr">
+      <c r="C80" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D78" s="13" t="inlineStr">
+      <c r="D80" s="13" t="inlineStr">
         <is>
           <t>Understanding the universe with weak lensing</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4039,24 +4129,24 @@
           </r>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
+      <c r="B81" s="4" t="inlineStr">
         <is>
           <t>2005</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
+      <c r="C81" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D79" s="5" t="inlineStr">
+      <c r="D81" s="5" t="inlineStr">
         <is>
           <t>Star Formation Efficiency and the Life Cycle of Molecular Clouds</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="14" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4084,24 +4174,24 @@
           </r>
         </is>
       </c>
-      <c r="B80" s="14" t="inlineStr">
+      <c r="B82" s="14" t="inlineStr">
         <is>
           <t>2005</t>
         </is>
       </c>
-      <c r="C80" s="14" t="inlineStr">
+      <c r="C82" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D80" s="15" t="inlineStr">
+      <c r="D82" s="15" t="inlineStr">
         <is>
           <t>The Evolution of Neutral Gas from the Epoch of Reionization to the Present</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="16" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4129,24 +4219,24 @@
           </r>
         </is>
       </c>
-      <c r="B81" s="16" t="inlineStr">
+      <c r="B83" s="16" t="inlineStr">
         <is>
           <t>2004</t>
         </is>
       </c>
-      <c r="C81" s="16" t="inlineStr">
+      <c r="C83" s="16" t="inlineStr">
         <is>
           <t>Exoplanet Formation and Protoplanetary Disks</t>
         </is>
       </c>
-      <c r="D81" s="17" t="inlineStr">
+      <c r="D83" s="17" t="inlineStr">
         <is>
           <t>(unspecified title)</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="12" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4174,24 +4264,24 @@
           </r>
         </is>
       </c>
-      <c r="B82" s="12" t="inlineStr">
+      <c r="B84" s="12" t="inlineStr">
         <is>
           <t>2004</t>
         </is>
       </c>
-      <c r="C82" s="12" t="inlineStr">
+      <c r="C84" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D82" s="13" t="inlineStr">
+      <c r="D84" s="13" t="inlineStr">
         <is>
           <t>Constraining Fundamental Physics Using the Cosmic Microwave Background and Complementary Data</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="14" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4219,109 +4309,19 @@
           </r>
         </is>
       </c>
-      <c r="B83" s="14" t="inlineStr">
+      <c r="B85" s="14" t="inlineStr">
         <is>
           <t>2003</t>
         </is>
       </c>
-      <c r="C83" s="14" t="inlineStr">
+      <c r="C85" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D83" s="15" t="inlineStr">
+      <c r="D85" s="15" t="inlineStr">
         <is>
           <t>The Nature and Origin of Dwarf Elliptical Galaxies</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Jeffrey Newman</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B84" s="14" t="inlineStr">
-        <is>
-          <t>2003</t>
-        </is>
-      </c>
-      <c r="C84" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D84" s="15" t="inlineStr">
-        <is>
-          <t>(unspecified title)</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Jason Aufdenberg</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00b30219"/>
-            </rPr>
-            <t>Michelson</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>2003</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>Stellar Physics</t>
-        </is>
-      </c>
-      <c r="D85" s="5" t="inlineStr">
-        <is>
-          <t>21st Century Interferometry of Hot Star Photospheres</t>
         </is>
       </c>
     </row>
@@ -4332,7 +4332,7 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Martin Bureau</t>
+            <t>Jeffrey Newman</t>
           </r>
           <r>
             <rPr>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="C86" s="14" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="D86" s="15" t="inlineStr">
         <is>
-          <t>Galactic Dynamics Over 4 Orders of Magnitude in Radii</t>
+          <t>(unspecified title)</t>
         </is>
       </c>
     </row>
@@ -4377,19 +4377,19 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Keivan Stassun</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
+            <t>Jason Aufdenberg</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00b30219"/>
+            </rPr>
+            <t>Michelson</t>
           </r>
           <r>
             <rPr>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Observational Tests of Pre-Main-Sequence Stellar Evolution Theory</t>
+          <t>21st Century Interferometry of Hot Star Photospheres</t>
         </is>
       </c>
     </row>
@@ -4422,6 +4422,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Martin Bureau</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D88" s="15" t="inlineStr">
+        <is>
+          <t>Galactic Dynamics Over 4 Orders of Magnitude in Radii</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Keivan Stassun</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Stellar Physics</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Observational Tests of Pre-Main-Sequence Stellar Evolution Theory</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Andrew Hopkins</t>
           </r>
           <r>
@@ -4444,109 +4534,19 @@
           </r>
         </is>
       </c>
-      <c r="B88" s="14" t="inlineStr">
+      <c r="B90" s="14" t="inlineStr">
         <is>
           <t>2001</t>
         </is>
       </c>
-      <c r="C88" s="14" t="inlineStr">
+      <c r="C90" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D88" s="15" t="inlineStr">
+      <c r="D90" s="15" t="inlineStr">
         <is>
           <t>Evolution of star-forming galaxies spanning $0&lt;z\lesssim2$</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Jeremy Heyl</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="005f1b6b"/>
-            </rPr>
-            <t>Chandra</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>Compact Objects and Accretion</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>Probing the Physics of Neutron Stars Through Observations of their Atmospheres</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Chris Reynolds</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>1998</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>Compact Objects and Accretion</t>
-        </is>
-      </c>
-      <c r="D90" s="3" t="inlineStr">
-        <is>
-          <t>The Central Engines and Immediate Environments of Active Galactic Nuclei</t>
         </is>
       </c>
     </row>
@@ -4557,6 +4557,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Jeremy Heyl</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="005f1b6b"/>
+            </rPr>
+            <t>Chandra</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Compact Objects and Accretion</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Probing the Physics of Neutron Stars Through Observations of their Atmospheres</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Chris Reynolds</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Compact Objects and Accretion</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>The Central Engines and Immediate Environments of Active Galactic Nuclei</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Bryan Gaensler</t>
           </r>
           <r>
@@ -4579,24 +4669,24 @@
           </r>
         </is>
       </c>
-      <c r="B91" s="2" t="inlineStr">
+      <c r="B93" s="2" t="inlineStr">
         <is>
           <t>1998</t>
         </is>
       </c>
-      <c r="C91" s="2" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>Compact Objects and Accretion</t>
         </is>
       </c>
-      <c r="D91" s="3" t="inlineStr">
+      <c r="D93" s="3" t="inlineStr">
         <is>
           <t>Born with a Band: Neutron Stars and their Origins</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="14" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4624,17 +4714,17 @@
           </r>
         </is>
       </c>
-      <c r="B92" s="14" t="inlineStr">
+      <c r="B94" s="14" t="inlineStr">
         <is>
           <t>1993</t>
         </is>
       </c>
-      <c r="C92" s="14" t="inlineStr">
+      <c r="C94" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D92" s="15" t="inlineStr">
+      <c r="D94" s="15" t="inlineStr">
         <is>
           <t>Starburst Galaxies at $z&lt;1$</t>
         </is>
@@ -4733,6 +4823,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add apps: Viraj Karambelkar, Jason Hinkle
</commit_message>
<xml_diff>
--- a/nhfp-apps/nhfp-apps.xlsx
+++ b/nhfp-apps/nhfp-apps.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D94"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -642,7 +642,7 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Nicholas Rui</t>
+            <t>Viraj Karambelkar</t>
           </r>
           <r>
             <rPr>
@@ -676,7 +676,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>A seismic atlas of the stellar merger sky</t>
+          <t>The Anthropology of Merging Stars</t>
         </is>
       </c>
     </row>
@@ -687,6 +687,51 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Nicholas Rui</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Stellar Physics</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>A seismic atlas of the stellar merger sky</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Lindsey Kwok</t>
           </r>
           <r>
@@ -709,24 +754,24 @@
           </r>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Determining the Astrophysical Origins of White-Dwarf Supernovae with JWST Infrared Spectroscopy</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -754,24 +799,69 @@
           </r>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Compact Objects and Accretion</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>From Glimmering Jewels to Cosmic Ubiquity: Unraveling the Origins of FRBs</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Jason Hinkle</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Compact Objects and Accretion</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Nuclear Transients in the Golden Era of Time-Domain Astronomy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -799,24 +889,24 @@
           </r>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>The Milky Way and Resolved Stellar Populations</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Beyond Mg and Fe: Exploring Detailed Nucleosynthetic Patterns</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -844,24 +934,24 @@
           </r>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Final Moments: Uncovering the Rate of Enhanced Red Supergiant Mass-loss in the Local Volume</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -889,24 +979,24 @@
           </r>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Optimizing The Vector Field For Next-Generation Astrophysics</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -934,24 +1024,24 @@
           </r>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>The Milky Way and Resolved Stellar Populations</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Inferring Kinematic and Chemical Maps of Galactic Dust</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -979,24 +1069,24 @@
           </r>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>The Milky Way and Resolved Stellar Populations</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>A Portrait of the Triangulum: Advancing a New Frontier of Galaxy Evolution with Resolved Stars</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1024,109 +1114,19 @@
           </r>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Gravitational Wave Astrophysics</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>From black holes to the Big Bang: astrophysics and cosmology with gravitational waves and their electromagnetic counterparts</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Maggie Thompson</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>To Explore Strange New Worlds: Connecting the Interiors and Atmospheres of Rocky Exoplanets</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Justin Pierel</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>Physics and Cosmology</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>Leveraging HST for a New Era of Precision NIR SN Ia Cosmology</t>
         </is>
       </c>
     </row>
@@ -1137,6 +1137,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Maggie Thompson</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>To Explore Strange New Worlds: Connecting the Interiors and Atmospheres of Rocky Exoplanets</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Justin Pierel</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Physics and Cosmology</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Leveraging HST for a New Era of Precision NIR SN Ia Cosmology</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Adina Feinstein</t>
           </r>
           <r>
@@ -1159,24 +1249,24 @@
           </r>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>The Evolution of Young Exoplanet Atmospheres in the Presence of Extreme Stellar Activity</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1204,24 +1294,24 @@
           </r>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>Illuminating the Primeval Universe with Lyman$\alpha$</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1249,109 +1339,19 @@
           </r>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Constraining Post-main-sequence Angular Momentum Evolution with Mixed-mode Asteroseismology</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Dávid Guszejnov</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Stellar Physics</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>The Role of Physical Processes and the Environment in Star Formation</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Pradip Gatkine</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="inlineStr">
-        <is>
-          <t>Probing the CGM-galaxy connection using Multi-object Spectroscopy and Astrophotonics</t>
         </is>
       </c>
     </row>
@@ -1362,6 +1362,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Dávid Guszejnov</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Stellar Physics</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>The Role of Physical Processes and the Environment in Star Formation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Pradip Gatkine</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Probing the CGM-galaxy connection using Multi-object Spectroscopy and Astrophotonics</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Michael Grudić</t>
           </r>
           <r>
@@ -1384,24 +1474,24 @@
           </r>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Star-Formation Physics from Cosmos to Cores</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1429,24 +1519,24 @@
           </r>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Atmospheres as Windows to the Diversity of Extrasolar Planets</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1474,24 +1564,24 @@
           </r>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Internal Structure of Massive Elliptical Galaxies: The Missing Piece at the Intersection of Astrophysics and Cosmology</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1519,24 +1609,24 @@
           </r>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>Cosmic Ray Diffusion in the Multi-phase Interstellar Medium</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1564,109 +1654,19 @@
           </r>
         </is>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C24" s="16" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>Exoplanet Formation and Protoplanetary Disks</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>Formation and Dynamics of Short-Period Exoplanetary Systems</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Peter Gao</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>The Role of Aerosols in the Formation and Early Evolution of Giant Planets</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Michael Zevin</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>Gravitational Wave Astrophysics</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>Deciphering the Biography of Massive Stars: Compact Object Mergers as a Rosetta Stone</t>
         </is>
       </c>
     </row>
@@ -1677,6 +1677,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Peter Gao</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>The Role of Aerosols in the Formation and Early Evolution of Giant Planets</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Michael Zevin</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Gravitational Wave Astrophysics</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Deciphering the Biography of Massive Stars: Compact Object Mergers as a Rosetta Stone</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Kevin Wagner</t>
           </r>
           <r>
@@ -1699,109 +1789,19 @@
           </r>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>A New Era of Exoplanet Imaging Mid-Infrared Exploration of the Habitable Zones of Nearby Stars</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>David Martin</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Two Projects with Circumbinary Planets—Using the Planets to Solve Super-Earth Formation, and the Binaries to Empirically Constrain M-dwarfs</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>David Jones</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>Physics and Cosmology</t>
-        </is>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>Supernova Cosmology in the Era of Cosmological Tensions</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Arpita Roy</t>
+            <t>David Martin</t>
           </r>
           <r>
             <rPr>
@@ -1846,7 +1846,7 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Of Worlds to Come: Delivering On the Promise of Extreme Precision Spectroscopy for Exoplanets</t>
+          <t>Two Projects with Circumbinary Planets—Using the Planets to Solve Super-Earth Formation, and the Binaries to Empirically Constrain M-dwarfs</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1857,7 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Yao-Yuan Mao</t>
+            <t>David Jones</t>
           </r>
           <r>
             <rPr>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
@@ -1891,52 +1891,52 @@
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>The Galaxy–Halo Connection: Probing the Dark Universe with Galaxies</t>
+          <t>Supernova Cosmology in the Era of Cosmological Tensions</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Georgia Panopoulou</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>The Milky Way and Resolved Stellar Populations</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>A unique approach to the determination of the Galactic magnetic field using starlight and synchrotron polarization observations</t>
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Arpita Roy</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Of Worlds to Come: Delivering On the Promise of Extreme Precision Spectroscopy for Exoplanets</t>
         </is>
       </c>
     </row>
@@ -1947,7 +1947,7 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Dillon Brout</t>
+            <t>Yao-Yuan Mao</t>
           </r>
           <r>
             <rPr>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>Improving Cosmological Constraints with the Dark Energy Survey Supernova Program and a Decade of Type Ia Supernovae</t>
+          <t>The Galaxy–Halo Connection: Probing the Dark Universe with Galaxies</t>
         </is>
       </c>
     </row>
@@ -1992,6 +1992,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Georgia Panopoulou</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>The Milky Way and Resolved Stellar Populations</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>A unique approach to the determination of the Galactic magnetic field using starlight and synchrotron polarization observations</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Dillon Brout</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Physics and Cosmology</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Improving Cosmological Constraints with the Dark Energy Survey Supernova Program and a Decade of Type Ia Supernovae</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Coral Wheeler</t>
           </r>
           <r>
@@ -2014,24 +2104,24 @@
           </r>
         </is>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>The Milky Way and Resolved Stellar Populations</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>Ultra-High Resolution Simulations of the Milky Way and its Satellites</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2059,24 +2149,24 @@
           </r>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D37" s="9" t="inlineStr">
         <is>
           <t>Planetary Collisions around Low-Mass Stars: Constraining the Timescale for Collisions and Testing the Origin of the Kepler Dichotomy</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2104,24 +2194,24 @@
           </r>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>Subgiants: Models, Rotation, Convection, and Planets</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="14" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2149,24 +2239,24 @@
           </r>
         </is>
       </c>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr">
+      <c r="C39" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="D39" s="15" t="inlineStr">
         <is>
           <t>Revolutionizing Reionization with JWST</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="14" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2194,24 +2284,24 @@
           </r>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
+      <c r="C40" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D38" s="15" t="inlineStr">
+      <c r="D40" s="15" t="inlineStr">
         <is>
           <t>Mapping the true boundary of dark matter halos with the splashback radius</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="12" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2239,24 +2329,24 @@
           </r>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="C39" s="12" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D39" s="13" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>The Role of Neutral‐ion Coupling in Star Formation</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2284,109 +2374,19 @@
           </r>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="D42" s="9" t="inlineStr">
         <is>
           <t>Breaking the Ultimate Barrier to Characterizing Other Earths</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Johanna Teske</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>Characterizing the Diversity of Small Planet Compositions via Planet Densities and Host Star Abundances</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Brett McGuire</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>The Milky Way and Resolved Stellar Populations</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>Getting Away from One-Pot Syntheses: Heterogeneity in Molecular Evolution Revealed with ALMA</t>
         </is>
       </c>
     </row>
@@ -2397,6 +2397,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Johanna Teske</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Characterizing the Diversity of Small Planet Compositions via Planet Densities and Host Star Abundances</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Brett McGuire</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>The Milky Way and Resolved Stellar Populations</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Getting Away from One-Pot Syntheses: Heterogeneity in Molecular Evolution Revealed with ALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Andrew Vanderburg</t>
           </r>
           <r>
@@ -2419,24 +2509,24 @@
           </r>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C45" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D45" s="9" t="inlineStr">
         <is>
           <t>The Galactic Distribution of Exoplanets</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="14" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2464,24 +2554,24 @@
           </r>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="C44" s="14" t="inlineStr">
+      <c r="C46" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>Unveiling the relationship between AGN and the CGM: feeding and feedback</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2509,24 +2599,24 @@
           </r>
         </is>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>The Milky Way and Resolved Stellar Populations</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>Bringing the Galactic Center into focus with dust scattering</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2554,24 +2644,24 @@
           </r>
         </is>
       </c>
-      <c r="B46" s="16" t="inlineStr">
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="C46" s="16" t="inlineStr">
+      <c r="C48" s="16" t="inlineStr">
         <is>
           <t>Exoplanet Formation and Protoplanetary Disks</t>
         </is>
       </c>
-      <c r="D46" s="17" t="inlineStr">
+      <c r="D48" s="17" t="inlineStr">
         <is>
           <t>Finding and Characterizing Forming Protoplanets with Next Generation Adaptive Optics Systems</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2599,24 +2689,24 @@
           </r>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>The Stellar Remnants of Double White Dwarf Mergers</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2644,109 +2734,19 @@
           </r>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>2016</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="D50" s="9" t="inlineStr">
         <is>
           <t>Characterizing Small Planets Around Bright Stars</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Tyler Robinson</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D49" s="9" t="inlineStr">
-        <is>
-          <t>Bridging the Theory Gap: Developing a Novel Cloud Model for Exoplanets</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Peter Behroozi</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B50" s="14" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
-      <c r="C50" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D50" s="15" t="inlineStr">
-        <is>
-          <t>Uncovering Connections between Galaxy and Dark Matter Halo Assembly Histories</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Daniel Foreman-Mackey</t>
+            <t>Tyler Robinson</t>
           </r>
           <r>
             <rPr>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>(unspecified title)</t>
+          <t>Bridging the Theory Gap: Developing a Novel Cloud Model for Exoplanets</t>
         </is>
       </c>
     </row>
@@ -2802,6 +2802,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Peter Behroozi</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="inlineStr">
+        <is>
+          <t>Uncovering Connections between Galaxy and Dark Matter Halo Assembly Histories</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Daniel Foreman-Mackey</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>(unspecified title)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Brooke Simmons</t>
           </r>
           <r>
@@ -2824,24 +2914,24 @@
           </r>
         </is>
       </c>
-      <c r="B52" s="14" t="inlineStr">
+      <c r="B54" s="14" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="C52" s="14" t="inlineStr">
+      <c r="C54" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="D54" s="15" t="inlineStr">
         <is>
           <t>Illuminating the Black Hole-Galaxy Connection</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2869,109 +2959,19 @@
           </r>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="C53" s="12" t="inlineStr">
+      <c r="C55" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D53" s="13" t="inlineStr">
+      <c r="D55" s="13" t="inlineStr">
         <is>
           <t>From a Detection to Astrophysics in 21 cm Cosmology</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Matteo Brogi</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B54" s="8" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>Pushing forward the frontiers of exoplanet characterization</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>James Owen</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B55" s="16" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="C55" s="16" t="inlineStr">
-        <is>
-          <t>Exoplanet Formation and Protoplanetary Disks</t>
-        </is>
-      </c>
-      <c r="D55" s="17" t="inlineStr">
-        <is>
-          <t>Formation and evolution of exoplanets</t>
         </is>
       </c>
     </row>
@@ -2982,6 +2982,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Matteo Brogi</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>Pushing forward the frontiers of exoplanet characterization</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>James Owen</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Exoplanet Formation and Protoplanetary Disks</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>Formation and evolution of exoplanets</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Ian Crossfield</t>
           </r>
           <r>
@@ -3004,109 +3094,19 @@
           </r>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="C56" s="8" t="inlineStr">
+      <c r="C58" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D56" s="9" t="inlineStr">
+      <c r="D58" s="9" t="inlineStr">
         <is>
           <t>Spectroscopy and Cartography of Cool Extrasolar Atmospheres</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Grant Tremblay</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Compact Objects and Accretion</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>Unifying Chandra with ALMA: Star Formation amid Kinematic Black Hole Feedback</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="10" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Francois Foucart</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>Gravitational Wave Astrophysics</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="inlineStr">
-        <is>
-          <t>Simulating compact binary mergers for multi-messenger astronomy</t>
         </is>
       </c>
     </row>
@@ -3117,6 +3117,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Grant Tremblay</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Compact Objects and Accretion</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Unifying Chandra with ALMA: Star Formation amid Kinematic Black Hole Feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Francois Foucart</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>Gravitational Wave Astrophysics</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Simulating compact binary mergers for multi-messenger astronomy</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Krzysztof Nalewajko</t>
           </r>
           <r>
@@ -3139,109 +3229,19 @@
           </r>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Compact Objects and Accretion</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>Understanding Gamma-Ray Flares of Blazars</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Jonathan Trump</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B60" s="14" t="inlineStr">
-        <is>
-          <t>2013</t>
-        </is>
-      </c>
-      <c r="C60" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D60" s="15" t="inlineStr">
-        <is>
-          <t>The Physics Behind Galaxy / Black Hole Coevolution</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Laura Blecha</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B61" s="14" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="C61" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D61" s="15" t="inlineStr">
-        <is>
-          <t>Seeking the Origins of Single and Double Active Black Holes</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,52 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Julie Hlavacek-Larrondo</t>
+            <t>Jonathan Trump</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>The Physics Behind Galaxy / Black Hole Coevolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Laura Blecha</t>
           </r>
           <r>
             <rPr>
@@ -3274,64 +3319,19 @@
           </r>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>2012</t>
         </is>
       </c>
-      <c r="C62" s="14" t="inlineStr">
+      <c r="C63" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D62" s="15" t="inlineStr">
-        <is>
-          <t>Unravelling AGN feedback: from isolated elliptical galaxies to massive clusters of galaxies</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Ann-Marie Madigan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00be006c"/>
-            </rPr>
-            <t>Einstein</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>Stellar Physics</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>The dynamics of stars in disks around massive black holes</t>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>Seeking the Origins of Single and Double Active Black Holes</t>
         </is>
       </c>
     </row>
@@ -3342,6 +3342,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Julie Hlavacek-Larrondo</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>Unravelling AGN feedback: from isolated elliptical galaxies to massive clusters of galaxies</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Ann-Marie Madigan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00be006c"/>
+            </rPr>
+            <t>Einstein</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Stellar Physics</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>The dynamics of stars in disks around massive black holes</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Steven Finkelstein</t>
           </r>
           <r>
@@ -3364,24 +3454,24 @@
           </r>
         </is>
       </c>
-      <c r="B64" s="14" t="inlineStr">
+      <c r="B66" s="14" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C64" s="14" t="inlineStr">
+      <c r="C66" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D64" s="15" t="inlineStr">
+      <c r="D66" s="15" t="inlineStr">
         <is>
           <t>Measuring the Evolution of Galaxy Physical Properties from z = 2 – 8</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3409,24 +3499,24 @@
           </r>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>Compact Objects and Accretion</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
+      <c r="D67" s="3" t="inlineStr">
         <is>
           <t>Probing extremes of binary evolution using subluminous X-ray binaries</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3454,24 +3544,24 @@
           </r>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>Compact Objects and Accretion</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>Theoretical Investigations of Type Ia Supernova Progenitors</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="16" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3499,24 +3589,24 @@
           </r>
         </is>
       </c>
-      <c r="B67" s="16" t="inlineStr">
+      <c r="B69" s="16" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C67" s="16" t="inlineStr">
+      <c r="C69" s="16" t="inlineStr">
         <is>
           <t>Exoplanet Formation and Protoplanetary Disks</t>
         </is>
       </c>
-      <c r="D67" s="17" t="inlineStr">
+      <c r="D69" s="17" t="inlineStr">
         <is>
           <t>The Formation and Structure of Proto-Planetary Disks Around the Youngest Protostars</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3544,24 +3634,24 @@
           </r>
         </is>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="C68" s="8" t="inlineStr">
+      <c r="C70" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D68" s="9" t="inlineStr">
+      <c r="D70" s="9" t="inlineStr">
         <is>
           <t>A Search for Exomoons</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="14" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3589,24 +3679,24 @@
           </r>
         </is>
       </c>
-      <c r="B69" s="14" t="inlineStr">
+      <c r="B71" s="14" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="C69" s="14" t="inlineStr">
+      <c r="C71" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D69" s="15" t="inlineStr">
+      <c r="D71" s="15" t="inlineStr">
         <is>
           <t>Revealing Cluster Astrophysics and Evolution with MUSTANG</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="12" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3634,24 +3724,24 @@
           </r>
         </is>
       </c>
-      <c r="B70" s="12" t="inlineStr">
+      <c r="B72" s="12" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="C70" s="12" t="inlineStr">
+      <c r="C72" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D70" s="13" t="inlineStr">
+      <c r="D72" s="13" t="inlineStr">
         <is>
           <t>Exploiting Gravitational Wave Observations: Modeling of Extreme-Mass Ratio Inspirals and Tests of Fundamental Physics</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3679,24 +3769,24 @@
           </r>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B73" s="8" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="C71" s="8" t="inlineStr">
+      <c r="C73" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D71" s="9" t="inlineStr">
+      <c r="D73" s="9" t="inlineStr">
         <is>
           <t>(unspecified title)</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3724,24 +3814,24 @@
           </r>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B74" s="8" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="C72" s="8" t="inlineStr">
+      <c r="C74" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D72" s="9" t="inlineStr">
+      <c r="D74" s="9" t="inlineStr">
         <is>
           <t>Dynamical Architecture of Planetary Systems</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3769,109 +3859,19 @@
           </r>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B75" s="4" t="inlineStr">
         <is>
           <t>2009</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C75" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>The Angular Diameters and Physical Properties of Low-Mass Stars</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Shelley Wright</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B74" s="14" t="inlineStr">
-        <is>
-          <t>2009</t>
-        </is>
-      </c>
-      <c r="C74" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D74" s="15" t="inlineStr">
-        <is>
-          <t>Galactic Disk Formation, AGN, and Metallicity in the Early Universe: Spatially Resolved Spectroscopy of High-Redshift Galaxies</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Kristian Finlator</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B75" s="14" t="inlineStr">
-        <is>
-          <t>2009</t>
-        </is>
-      </c>
-      <c r="C75" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D75" s="15" t="inlineStr">
-        <is>
-          <t>Radiative Hydrodynamic Simulations of Galaxies in the Reionization Epoch</t>
         </is>
       </c>
     </row>
@@ -3882,6 +3882,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Shelley Wright</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>Galactic Disk Formation, AGN, and Metallicity in the Early Universe: Spatially Resolved Spectroscopy of High-Redshift Galaxies</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Kristian Finlator</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D77" s="15" t="inlineStr">
+        <is>
+          <t>Radiative Hydrodynamic Simulations of Galaxies in the Reionization Epoch</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>John Wise</t>
           </r>
           <r>
@@ -3904,109 +3994,19 @@
           </r>
         </is>
       </c>
-      <c r="B76" s="14" t="inlineStr">
+      <c r="B78" s="14" t="inlineStr">
         <is>
           <t>2009</t>
         </is>
       </c>
-      <c r="C76" s="14" t="inlineStr">
+      <c r="C78" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D76" s="15" t="inlineStr">
+      <c r="D78" s="15" t="inlineStr">
         <is>
           <t>Ab Initio Dwarf Galaxy Formation – Predictions for JWST and ALMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Eliza Kempton</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00cf9306"/>
-            </rPr>
-            <t>Sagan</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B77" s="8" t="inlineStr">
-        <is>
-          <t>2009</t>
-        </is>
-      </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t>Exoplanets and Habitability</t>
-        </is>
-      </c>
-      <c r="D77" s="9" t="inlineStr">
-        <is>
-          <t>(unspecified title)</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Kelle Cruz</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00fa4224"/>
-            </rPr>
-            <t>Spitzer</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>2007</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>Stellar Physics</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>Nearby, Young Brown Dwarfs: A Comprehensive Study</t>
         </is>
       </c>
     </row>
@@ -4017,6 +4017,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Eliza Kempton</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00cf9306"/>
+            </rPr>
+            <t>Sagan</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>Exoplanets and Habitability</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>(unspecified title)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Kelle Cruz</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00fa4224"/>
+            </rPr>
+            <t>Spitzer</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Stellar Physics</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Nearby, Young Brown Dwarfs: A Comprehensive Study</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Daniel Fabrycky</t>
           </r>
           <r>
@@ -4039,24 +4129,24 @@
           </r>
         </is>
       </c>
-      <c r="B79" s="8" t="inlineStr">
+      <c r="B81" s="8" t="inlineStr">
         <is>
           <t>2007</t>
         </is>
       </c>
-      <c r="C79" s="8" t="inlineStr">
+      <c r="C81" s="8" t="inlineStr">
         <is>
           <t>Exoplanets and Habitability</t>
         </is>
       </c>
-      <c r="D79" s="9" t="inlineStr">
+      <c r="D81" s="9" t="inlineStr">
         <is>
           <t>Dynamical detection and migration of multiple-body planetary systems</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="12" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4084,24 +4174,24 @@
           </r>
         </is>
       </c>
-      <c r="B80" s="12" t="inlineStr">
+      <c r="B82" s="12" t="inlineStr">
         <is>
           <t>2006</t>
         </is>
       </c>
-      <c r="C80" s="12" t="inlineStr">
+      <c r="C82" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D80" s="13" t="inlineStr">
+      <c r="D82" s="13" t="inlineStr">
         <is>
           <t>Understanding the universe with weak lensing</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="4" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4129,24 +4219,24 @@
           </r>
         </is>
       </c>
-      <c r="B81" s="4" t="inlineStr">
+      <c r="B83" s="4" t="inlineStr">
         <is>
           <t>2005</t>
         </is>
       </c>
-      <c r="C81" s="4" t="inlineStr">
+      <c r="C83" s="4" t="inlineStr">
         <is>
           <t>Stellar Physics</t>
         </is>
       </c>
-      <c r="D81" s="5" t="inlineStr">
+      <c r="D83" s="5" t="inlineStr">
         <is>
           <t>Star Formation Efficiency and the Life Cycle of Molecular Clouds</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="14" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4174,24 +4264,24 @@
           </r>
         </is>
       </c>
-      <c r="B82" s="14" t="inlineStr">
+      <c r="B84" s="14" t="inlineStr">
         <is>
           <t>2005</t>
         </is>
       </c>
-      <c r="C82" s="14" t="inlineStr">
+      <c r="C84" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D82" s="15" t="inlineStr">
+      <c r="D84" s="15" t="inlineStr">
         <is>
           <t>The Evolution of Neutral Gas from the Epoch of Reionization to the Present</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="16" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4219,24 +4309,24 @@
           </r>
         </is>
       </c>
-      <c r="B83" s="16" t="inlineStr">
+      <c r="B85" s="16" t="inlineStr">
         <is>
           <t>2004</t>
         </is>
       </c>
-      <c r="C83" s="16" t="inlineStr">
+      <c r="C85" s="16" t="inlineStr">
         <is>
           <t>Exoplanet Formation and Protoplanetary Disks</t>
         </is>
       </c>
-      <c r="D83" s="17" t="inlineStr">
+      <c r="D85" s="17" t="inlineStr">
         <is>
           <t>(unspecified title)</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="12" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="12" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4264,24 +4354,24 @@
           </r>
         </is>
       </c>
-      <c r="B84" s="12" t="inlineStr">
+      <c r="B86" s="12" t="inlineStr">
         <is>
           <t>2004</t>
         </is>
       </c>
-      <c r="C84" s="12" t="inlineStr">
+      <c r="C86" s="12" t="inlineStr">
         <is>
           <t>Physics and Cosmology</t>
         </is>
       </c>
-      <c r="D84" s="13" t="inlineStr">
+      <c r="D86" s="13" t="inlineStr">
         <is>
           <t>Constraining Fundamental Physics Using the Cosmic Microwave Background and Complementary Data</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="14" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4309,109 +4399,19 @@
           </r>
         </is>
       </c>
-      <c r="B85" s="14" t="inlineStr">
+      <c r="B87" s="14" t="inlineStr">
         <is>
           <t>2003</t>
         </is>
       </c>
-      <c r="C85" s="14" t="inlineStr">
+      <c r="C87" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D85" s="15" t="inlineStr">
+      <c r="D87" s="15" t="inlineStr">
         <is>
           <t>The Nature and Origin of Dwarf Elliptical Galaxies</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="14" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Jeffrey Newman</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B86" s="14" t="inlineStr">
-        <is>
-          <t>2003</t>
-        </is>
-      </c>
-      <c r="C86" s="14" t="inlineStr">
-        <is>
-          <t>Galaxies and the Intergalactic Medium</t>
-        </is>
-      </c>
-      <c r="D86" s="15" t="inlineStr">
-        <is>
-          <t>(unspecified title)</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Jason Aufdenberg</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00b30219"/>
-            </rPr>
-            <t>Michelson</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B87" s="4" t="inlineStr">
-        <is>
-          <t>2003</t>
-        </is>
-      </c>
-      <c r="C87" s="4" t="inlineStr">
-        <is>
-          <t>Stellar Physics</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>21st Century Interferometry of Hot Star Photospheres</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Martin Bureau</t>
+            <t>Jeffrey Newman</t>
           </r>
           <r>
             <rPr>
@@ -4446,7 +4446,7 @@
       </c>
       <c r="B88" s="14" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="C88" s="14" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="D88" s="15" t="inlineStr">
         <is>
-          <t>Galactic Dynamics Over 4 Orders of Magnitude in Radii</t>
+          <t>(unspecified title)</t>
         </is>
       </c>
     </row>
@@ -4467,19 +4467,19 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
-            <t>Keivan Stassun</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
+            <t>Jason Aufdenberg</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00b30219"/>
+            </rPr>
+            <t>Michelson</t>
           </r>
           <r>
             <rPr>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>Observational Tests of Pre-Main-Sequence Stellar Evolution Theory</t>
+          <t>21st Century Interferometry of Hot Star Photospheres</t>
         </is>
       </c>
     </row>
@@ -4512,6 +4512,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Martin Bureau</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>Galaxies and the Intergalactic Medium</t>
+        </is>
+      </c>
+      <c r="D90" s="15" t="inlineStr">
+        <is>
+          <t>Galactic Dynamics Over 4 Orders of Magnitude in Radii</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Keivan Stassun</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Stellar Physics</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Observational Tests of Pre-Main-Sequence Stellar Evolution Theory</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Andrew Hopkins</t>
           </r>
           <r>
@@ -4534,109 +4624,19 @@
           </r>
         </is>
       </c>
-      <c r="B90" s="14" t="inlineStr">
+      <c r="B92" s="14" t="inlineStr">
         <is>
           <t>2001</t>
         </is>
       </c>
-      <c r="C90" s="14" t="inlineStr">
+      <c r="C92" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D90" s="15" t="inlineStr">
+      <c r="D92" s="15" t="inlineStr">
         <is>
           <t>Evolution of star-forming galaxies spanning $0&lt;z\lesssim2$</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Jeremy Heyl</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="005f1b6b"/>
-            </rPr>
-            <t>Chandra</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>Compact Objects and Accretion</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr">
-        <is>
-          <t>Probing the Physics of Neutron Stars Through Observations of their Atmospheres</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>Chris Reynolds</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t xml:space="preserve"> (</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="008f1402"/>
-            </rPr>
-            <t>Hubble</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="00000000"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>1998</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>Compact Objects and Accretion</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>The Central Engines and Immediate Environments of Active Galactic Nuclei</t>
         </is>
       </c>
     </row>
@@ -4647,6 +4647,96 @@
             <rPr>
               <color rgb="00000000"/>
             </rPr>
+            <t>Jeremy Heyl</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="005f1b6b"/>
+            </rPr>
+            <t>Chandra</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Compact Objects and Accretion</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Probing the Physics of Neutron Stars Through Observations of their Atmospheres</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>Chris Reynolds</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="008f1402"/>
+            </rPr>
+            <t>Hubble</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Compact Objects and Accretion</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>The Central Engines and Immediate Environments of Active Galactic Nuclei</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="00000000"/>
+            </rPr>
             <t>Bryan Gaensler</t>
           </r>
           <r>
@@ -4669,24 +4759,24 @@
           </r>
         </is>
       </c>
-      <c r="B93" s="2" t="inlineStr">
+      <c r="B95" s="2" t="inlineStr">
         <is>
           <t>1998</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr">
+      <c r="C95" s="2" t="inlineStr">
         <is>
           <t>Compact Objects and Accretion</t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr">
+      <c r="D95" s="3" t="inlineStr">
         <is>
           <t>Born with a Band: Neutron Stars and their Origins</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="14" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4714,17 +4804,17 @@
           </r>
         </is>
       </c>
-      <c r="B94" s="14" t="inlineStr">
+      <c r="B96" s="14" t="inlineStr">
         <is>
           <t>1993</t>
         </is>
       </c>
-      <c r="C94" s="14" t="inlineStr">
+      <c r="C96" s="14" t="inlineStr">
         <is>
           <t>Galaxies and the Intergalactic Medium</t>
         </is>
       </c>
-      <c r="D94" s="15" t="inlineStr">
+      <c r="D96" s="15" t="inlineStr">
         <is>
           <t>Starburst Galaxies at $z&lt;1$</t>
         </is>
@@ -4825,6 +4915,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId95"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>